<commit_message>
updates output files again
</commit_message>
<xml_diff>
--- a/Altium/Project Outputs for UZ_PER_SKAI3_LV_48V_410A/Rev01/BOM/BOM_JLC-UZ_PER_SKAI3_LV_48V_410A.xlsx
+++ b/Altium/Project Outputs for UZ_PER_SKAI3_LV_48V_410A/Rev01/BOM/BOM_JLC-UZ_PER_SKAI3_LV_48V_410A.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\UltraZohm\uz_per_skai3_lv_48v_410a\Altium\Project Outputs for UZ_PER_SKAI3_LV_48V_410A\Rev01\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B9B15814-D4F6-4FE0-B0B7-80037DAAA464}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D94D7F89-FE2F-4416-A496-65E0455F9350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-29184" yWindow="1536" windowWidth="23040" windowHeight="12120" xr2:uid="{2CDE2C65-CF96-478A-BAA3-93C16F2DF380}"/>
+    <workbookView xWindow="-29184" yWindow="1536" windowWidth="23040" windowHeight="12120" xr2:uid="{EFE41E5C-810B-4737-B31F-30E9A292824E}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC-UZ_PER_SKAI3_LV_48V_410" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="199">
   <si>
     <t>Quantity</t>
   </si>
@@ -500,7 +500,7 @@
     <t>5.05k</t>
   </si>
   <si>
-    <t>R29, R35A, R35B, R35C, R36A, R36B, R36C</t>
+    <t>R29, R35A, R35B, R35C, R36A, R36B, R36C, R49, R50</t>
   </si>
   <si>
     <t>Vishay</t>
@@ -510,15 +510,6 @@
   </si>
   <si>
     <t>C1693738</t>
-  </si>
-  <si>
-    <t>R49, R50</t>
-  </si>
-  <si>
-    <t>TNPW04025K05BEED</t>
-  </si>
-  <si>
-    <t>C4292536</t>
   </si>
   <si>
     <t>Serial #</t>
@@ -1040,8 +1031,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D9EF559-A98B-4F48-9012-470D4A584E38}">
-  <dimension ref="A1:K37"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C3935C8-525B-4E74-9142-3BBA2BCC14E3}">
+  <dimension ref="A1:K36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.44140625" customWidth="1"/>
@@ -1862,7 +1853,7 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>152</v>
@@ -1893,115 +1884,111 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>152</v>
-      </c>
+        <v>159</v>
+      </c>
+      <c r="E28" s="1"/>
       <c r="F28" s="2" t="s">
-        <v>127</v>
+        <v>160</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>107</v>
+        <v>161</v>
       </c>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
       <c r="J28" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="K28" s="2" t="s">
-        <v>159</v>
-      </c>
+        <v>162</v>
+      </c>
+      <c r="K28" s="1"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="E29" s="1"/>
       <c r="F29" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
       <c r="J29" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="K29" s="1"/>
+        <v>163</v>
+      </c>
+      <c r="K29" s="2" t="s">
+        <v>168</v>
+      </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="E30" s="1"/>
       <c r="F30" s="2" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="H30" s="1"/>
       <c r="I30" s="1"/>
       <c r="J30" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="K30" s="2" t="s">
-        <v>171</v>
-      </c>
+        <v>169</v>
+      </c>
+      <c r="K30" s="1"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>1</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="E31" s="1"/>
       <c r="F31" s="2" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
       <c r="J31" s="2" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="K31" s="1"/>
     </row>
@@ -2010,31 +1997,33 @@
         <v>1</v>
       </c>
       <c r="B32" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="C32" s="2" t="s">
-        <v>178</v>
-      </c>
       <c r="D32" s="2" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="E32" s="1"/>
       <c r="F32" s="2" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="H32" s="1"/>
       <c r="I32" s="1"/>
       <c r="J32" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="K32" s="1"/>
+        <v>176</v>
+      </c>
+      <c r="K32" s="2" t="s">
+        <v>178</v>
+      </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>179</v>
@@ -2043,14 +2032,14 @@
         <v>180</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="E33" s="1"/>
       <c r="F33" s="2" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="H33" s="1"/>
       <c r="I33" s="1"/>
@@ -2058,36 +2047,36 @@
         <v>179</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="E34" s="1"/>
       <c r="F34" s="2" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>186</v>
+        <v>167</v>
       </c>
       <c r="H34" s="1"/>
       <c r="I34" s="1"/>
       <c r="J34" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.3">
@@ -2095,83 +2084,54 @@
         <v>1</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>168</v>
+        <v>191</v>
       </c>
       <c r="E35" s="1"/>
       <c r="F35" s="2" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>170</v>
+        <v>193</v>
       </c>
       <c r="H35" s="1"/>
       <c r="I35" s="1"/>
       <c r="J35" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="K35" s="2" t="s">
-        <v>191</v>
-      </c>
+        <v>189</v>
+      </c>
+      <c r="K35" s="1"/>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="E36" s="1"/>
       <c r="F36" s="2" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="H36" s="1"/>
       <c r="I36" s="1"/>
       <c r="J36" s="2" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="K36" s="1"/>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A37" s="1">
-        <v>2</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="E37" s="1"/>
-      <c r="F37" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="G37" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="H37" s="1"/>
-      <c r="I37" s="1"/>
-      <c r="J37" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="K37" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Increases via hole size to min 0.3mm
</commit_message>
<xml_diff>
--- a/Altium/Project Outputs for UZ_PER_SKAI3_LV_48V_410A/Rev01/BOM/BOM_JLC-UZ_PER_SKAI3_LV_48V_410A.xlsx
+++ b/Altium/Project Outputs for UZ_PER_SKAI3_LV_48V_410A/Rev01/BOM/BOM_JLC-UZ_PER_SKAI3_LV_48V_410A.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\UltraZohm\uz_per_skai3_lv_48v_410a\Altium\Project Outputs for UZ_PER_SKAI3_LV_48V_410A\Rev01\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D94D7F89-FE2F-4416-A496-65E0455F9350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D8472E1C-71AC-4234-89F4-A505EBF6861A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-29184" yWindow="1536" windowWidth="23040" windowHeight="12120" xr2:uid="{EFE41E5C-810B-4737-B31F-30E9A292824E}"/>
+    <workbookView xWindow="-29184" yWindow="1536" windowWidth="23040" windowHeight="12120" xr2:uid="{95FBE25B-CCFD-455D-A9FE-13477F97A1CA}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC-UZ_PER_SKAI3_LV_48V_410" sheetId="1" r:id="rId1"/>
@@ -1031,7 +1031,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C3935C8-525B-4E74-9142-3BBA2BCC14E3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67837F8C-34AE-472F-BB1C-379D3F28434D}">
   <dimension ref="A1:K36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>

</xml_diff>

<commit_message>
Fixes all 100nF caps to the same part
</commit_message>
<xml_diff>
--- a/Altium/Project Outputs for UZ_PER_SKAI3_LV_48V_410A/Rev01/BOM/BOM_JLC-UZ_PER_SKAI3_LV_48V_410A.xlsx
+++ b/Altium/Project Outputs for UZ_PER_SKAI3_LV_48V_410A/Rev01/BOM/BOM_JLC-UZ_PER_SKAI3_LV_48V_410A.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\UltraZohm\uz_per_skai3_lv_48v_410a\Altium\Project Outputs for UZ_PER_SKAI3_LV_48V_410A\Rev01\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8CC462E6-E986-4558-9DAF-57677B05A406}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{15F2D015-7133-4D89-BDAB-0DA334A1D03A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-29184" yWindow="1536" windowWidth="23040" windowHeight="12120" xr2:uid="{4587B08F-1754-49E6-A3BD-52B8FBFCA577}"/>
+    <workbookView xWindow="-28836" yWindow="1884" windowWidth="23040" windowHeight="12120" xr2:uid="{5893EC66-36C4-4960-AE19-70A0ECC6D802}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC-UZ_PER_SKAI3_LV_48V_410" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="193">
   <si>
     <t>Quantity</t>
   </si>
@@ -77,7 +77,7 @@
     <t>0.1 µF</t>
   </si>
   <si>
-    <t>C1, C2, C6, C8, C10, C11, C12, C13, C19, C20, C21, C22, C29A, C29B, C29C, C31A, C31B, C31C, C38</t>
+    <t>C1, C2, C6, C8, C10, C11, C12, C13, C19, C20, C21, C22, C29A, C29B, C29C, C30A, C30B, C30C, C31A, C31B, C31C, C32A, C32B, C32C, C38</t>
   </si>
   <si>
     <t>KEMET</t>
@@ -198,24 +198,6 @@
   </si>
   <si>
     <t>C107185</t>
-  </si>
-  <si>
-    <t>100 nF</t>
-  </si>
-  <si>
-    <t>C30A, C30B, C30C, C32A, C32B, C32C</t>
-  </si>
-  <si>
-    <t>TDK</t>
-  </si>
-  <si>
-    <t>100V 100nF X7S ±10% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
-  </si>
-  <si>
-    <t>C1608X7S2A104KT000N</t>
-  </si>
-  <si>
-    <t>C343025</t>
   </si>
   <si>
     <t>150060GS84000</t>
@@ -1031,8 +1013,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD8B586C-93A0-484C-ADAC-CB7DED36473A}">
-  <dimension ref="A1:K36"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FBC74AA-126C-4DA6-B34E-B607072C555F}">
+  <dimension ref="A1:K35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.44140625" customWidth="1"/>
@@ -1084,7 +1066,7 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>11</v>
@@ -1301,7 +1283,7 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>53</v>
@@ -1313,26 +1295,26 @@
         <v>55</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>15</v>
+        <v>58</v>
       </c>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
       <c r="J9" s="2" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>59</v>
@@ -1357,13 +1339,11 @@
       <c r="J10" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="K10" s="2" t="s">
-        <v>62</v>
-      </c>
+      <c r="K10" s="1"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>65</v>
@@ -1374,49 +1354,51 @@
       <c r="D11" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" s="1"/>
+      <c r="F11" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="F11" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="G11" s="2" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
       <c r="J11" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="K11" s="1"/>
+      <c r="K11" s="2" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="E12" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E12" s="1"/>
       <c r="F12" s="2" t="s">
         <v>74</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
       <c r="J12" s="2" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
@@ -1424,22 +1406,22 @@
         <v>1</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
@@ -1452,7 +1434,7 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>84</v>
@@ -1461,38 +1443,38 @@
         <v>85</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
       <c r="J14" s="2" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>93</v>
@@ -1506,7 +1488,7 @@
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
       <c r="J15" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K15" s="2" t="s">
         <v>96</v>
@@ -1514,7 +1496,7 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>97</v>
@@ -1523,10 +1505,10 @@
         <v>98</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>100</v>
@@ -1537,95 +1519,95 @@
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
       <c r="J16" s="2" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C17" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="E17" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>103</v>
-      </c>
       <c r="F17" s="2" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
       <c r="J17" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="K17" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="K17" s="2" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="B18" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="C18" s="2" t="s">
-        <v>111</v>
-      </c>
       <c r="D18" s="2" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
       <c r="J18" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B19" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="E19" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="F19" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>106</v>
-      </c>
       <c r="G19" s="2" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
@@ -1647,244 +1629,240 @@
         <v>120</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>121</v>
+        <v>106</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>119</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
       <c r="J20" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="K20" s="2" t="s">
-        <v>124</v>
-      </c>
+        <v>122</v>
+      </c>
+      <c r="K20" s="1"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>127</v>
+        <v>100</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
       <c r="J21" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="K21" s="1"/>
+        <v>125</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>1</v>
       </c>
       <c r="B22" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="F22" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="C22" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>106</v>
-      </c>
       <c r="G22" s="2" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
       <c r="J22" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="K22" s="2" t="s">
         <v>131</v>
-      </c>
-      <c r="K22" s="2" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="C23" s="2" t="s">
-        <v>134</v>
-      </c>
       <c r="D23" s="2" t="s">
-        <v>44</v>
+        <v>106</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
       <c r="J23" s="2" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B24" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="C24" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>112</v>
-      </c>
       <c r="E24" s="2" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>135</v>
+        <v>121</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
       <c r="J24" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="K24" s="2" t="s">
         <v>140</v>
-      </c>
-      <c r="K24" s="2" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B25" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="D25" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="F25" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="D25" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>127</v>
-      </c>
       <c r="G25" s="2" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
       <c r="J25" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K25" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="K25" s="2" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B26" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="D26" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>105</v>
-      </c>
       <c r="E26" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>149</v>
+        <v>121</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="H26" s="1"/>
       <c r="I26" s="1"/>
       <c r="J26" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="K26" s="2" t="s">
         <v>150</v>
-      </c>
-      <c r="K26" s="2" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="B27" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="D27" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="E27" s="1"/>
+      <c r="F27" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="E27" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>127</v>
-      </c>
       <c r="G27" s="2" t="s">
-        <v>107</v>
+        <v>155</v>
       </c>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
       <c r="J27" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="K27" s="2" t="s">
         <v>156</v>
       </c>
+      <c r="K27" s="1"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>157</v>
@@ -1905,13 +1883,15 @@
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
       <c r="J28" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="K28" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="K28" s="1"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>163</v>
@@ -1934,34 +1914,32 @@
       <c r="J29" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="K29" s="2" t="s">
-        <v>168</v>
-      </c>
+      <c r="K29" s="1"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>1</v>
       </c>
       <c r="B30" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="C30" s="2" t="s">
-        <v>170</v>
-      </c>
       <c r="D30" s="2" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="E30" s="1"/>
       <c r="F30" s="2" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="H30" s="1"/>
       <c r="I30" s="1"/>
       <c r="J30" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="K30" s="1"/>
     </row>
@@ -1970,52 +1948,54 @@
         <v>1</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="E31" s="1"/>
       <c r="F31" s="2" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
       <c r="J31" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="K31" s="1"/>
+        <v>170</v>
+      </c>
+      <c r="K31" s="2" t="s">
+        <v>172</v>
+      </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="E32" s="1"/>
       <c r="F32" s="2" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="H32" s="1"/>
       <c r="I32" s="1"/>
       <c r="J32" s="2" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="K32" s="2" t="s">
         <v>178</v>
@@ -2023,7 +2003,7 @@
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>179</v>
@@ -2032,14 +2012,14 @@
         <v>180</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>181</v>
+        <v>159</v>
       </c>
       <c r="E33" s="1"/>
       <c r="F33" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>183</v>
+        <v>161</v>
       </c>
       <c r="H33" s="1"/>
       <c r="I33" s="1"/>
@@ -2047,7 +2027,7 @@
         <v>179</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.3">
@@ -2055,83 +2035,54 @@
         <v>1</v>
       </c>
       <c r="B34" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="D34" s="2" t="s">
         <v>185</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>165</v>
       </c>
       <c r="E34" s="1"/>
       <c r="F34" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="G34" s="2" t="s">
         <v>187</v>
-      </c>
-      <c r="G34" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="H34" s="1"/>
       <c r="I34" s="1"/>
       <c r="J34" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="K34" s="2" t="s">
-        <v>188</v>
-      </c>
+        <v>183</v>
+      </c>
+      <c r="K34" s="1"/>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B35" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="C35" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="C35" s="2" t="s">
+      <c r="D35" s="2" t="s">
         <v>190</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>191</v>
       </c>
       <c r="E35" s="1"/>
       <c r="F35" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="G35" s="2" t="s">
         <v>192</v>
-      </c>
-      <c r="G35" s="2" t="s">
-        <v>193</v>
       </c>
       <c r="H35" s="1"/>
       <c r="I35" s="1"/>
       <c r="J35" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="K35" s="1"/>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A36" s="1">
-        <v>2</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="E36" s="1"/>
-      <c r="F36" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="G36" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="H36" s="1"/>
-      <c r="I36" s="1"/>
-      <c r="J36" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="K36" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>